<commit_message>
Refine SCIE paper draft and evaluation outputs
</commit_message>
<xml_diff>
--- a/SCIE용/excel/30_g4_auto_retrieval_results.xlsx
+++ b/SCIE용/excel/30_g4_auto_retrieval_results.xlsx
@@ -130,7 +130,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>자동 G4 적용</t>
+          <t>G4 적용</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -1224,12 +1224,12 @@
 2. page_179_img_1_0.jpeg | score=1.297 | stage=0.698 | page=1.00; keyword=backdrive,recovery; section=backdrive
 3. page_181_img_0_0.jpeg | score=0.986 | stage=0.614 | page=1.00; keyword=recovery
 4. page_89_img_1_0.jpeg | score=0.899 | stage=0.341 | 
-5. page_177_img_1_0.jpeg | score=0.862 | stage=0.580 | page=1.00
+5. page_177_img_1_0.jpeg | score=0.864 | stage=0.580 | page=1.00
 6. page_125_img_0_0.jpeg | score=0.859 | stage=0.328 | 
 7. page_89_img_0_0.jpeg | score=0.840 | stage=0.337 | 
 8. page_24_img_0_0.jpeg | score=0.725 | stage=0.289 | keyword=emergency
-9. page_169_img_2_0.jpeg | score=0.709 | stage=0.698 | page=1.00; keyword=backdrive,recovery; section=backdrive
-10. page_174_img_1_0.jpeg | score=0.699 | stage=0.580 | page=1.00</t>
+9. page_169_img_2_0.jpeg | score=0.712 | stage=0.698 | page=1.00; keyword=backdrive,recovery; section=backdrive
+10. page_174_img_1_0.jpeg | score=0.701 | stage=0.580 | page=1.00</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
 6. page_330_img_0_0.jpeg | score=0.764 | stage=0.236 | 
 7. page_343_img_0_0.jpeg | score=0.745 | stage=0.651 | page=1.00; keyword=account; section=account
 8. page_147_img_0_0.jpeg | score=0.730 | stage=0.293 | 
-9. page_354_img_0_0.jpeg | score=0.680 | stage=0.580 | page=1.00
+9. page_354_img_0_0.jpeg | score=0.682 | stage=0.580 | page=1.00
 10. page_349_img_0_0.jpeg | score=0.647 | stage=0.647 | page=1.00; keyword=lock,setting</t>
         </is>
       </c>
@@ -5707,14 +5707,14 @@
       <c r="P63" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">1. page_196_img_0_0.jpeg | score=1.059 | stage=0.614 | page=1.00; keyword=setting
-2. page_195_img_2_0.jpeg | score=0.958 | stage=0.614 | page=1.00; keyword=setting
-3. page_192_img_0_0.jpeg | score=0.937 | stage=0.614 | page=1.00; keyword=setting
-4. page_190_img_1_0.jpeg | score=0.902 | stage=0.614 | page=1.00; keyword=setting
-5. page_190_img_0_0.jpeg | score=0.874 | stage=0.614 | page=1.00; keyword=setting
+2. page_195_img_2_0.jpeg | score=0.956 | stage=0.614 | page=1.00; keyword=setting
+3. page_192_img_0_0.jpeg | score=0.934 | stage=0.614 | page=1.00; keyword=setting
+4. page_190_img_1_0.jpeg | score=0.900 | stage=0.614 | page=1.00; keyword=setting
+5. page_190_img_0_0.jpeg | score=0.872 | stage=0.614 | page=1.00; keyword=setting
 6. page_220_img_0_0.jpeg | score=0.796 | stage=0.226 | keyword=setting
 7. page_224_img_0_0.jpeg | score=0.771 | stage=0.227 | keyword=setting
-8. page_195_img_0_0.jpeg | score=0.749 | stage=0.614 | page=1.00; keyword=setting
-9. page_376_img_0_0.jpeg | score=0.744 | stage=0.249 | 
+8. page_195_img_0_0.jpeg | score=0.746 | stage=0.614 | page=1.00; keyword=setting
+9. page_376_img_0_0.jpeg | score=0.742 | stage=0.245 | 
 10. page_235_img_1_0.jpeg | score=0.741 | stage=0.225 | keyword=setting</t>
         </is>
       </c>

</xml_diff>